<commit_message>
Correct VoCodec STFT latency accounting (#17)
</commit_message>
<xml_diff>
--- a/egs2/lrac2/track1/LRAC2-Track1-VoCodec-Model-Design-Sheet.xlsx
+++ b/egs2/lrac2/track1/LRAC2-Track1-VoCodec-Model-Design-Sheet.xlsx
@@ -885,7 +885,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>STFT buffering latency (ms)</t>
+          <t>Frame-hop buffering latency (ms)</t>
         </is>
       </c>
       <c r="B15" s="3">
@@ -1084,18 +1084,20 @@
         <f>C20*L20</f>
         <v/>
       </c>
-      <c r="N20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="6" t="n">
-        <v>0</v>
+      <c r="N20" s="6">
+        <f>($B$3-$B$4)/2</f>
+        <v/>
+      </c>
+      <c r="O20" s="6">
+        <f>($B$3-$B$4)/2</f>
+        <v/>
       </c>
       <c r="P20" s="8">
-        <f>C20*N20/$B$5*1000</f>
+        <f>C20*N20/$B$2*1000</f>
         <v/>
       </c>
       <c r="Q20" s="8">
-        <f>C20*O20/$B$5*1000</f>
+        <f>C20*O20/$B$2*1000</f>
         <v/>
       </c>
       <c r="R20" s="7">
@@ -2592,7 +2594,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Memory bandwidth uses the bytes-per-value setting in B16 and includes model parameters, model buffers, convolution state, and attention KV-cache. Parameter-cap values include trainable parameters and non-runtime model buffers required for inference. Runtime state/cache is excluded from the parameter cap, but its read/write traffic is included in memory bandwidth. Intermediate activations are excluded by the challenge convention. Attention MACs assume that the configured context buffer is fully populated; startup frames require less compute. FOV left is history, not latency; only FOV right contributes to algorithmic latency. STFT/ISTFT window and overlap-state bandwidth is shown explicitly in the first table row; FFT arithmetic is excluded.</t>
+          <t>Memory bandwidth uses the bytes-per-value setting in B16 and includes model parameters, model buffers, convolution state, and attention KV-cache. Parameter-cap values include trainable parameters and non-runtime model buffers required for inference. Runtime state/cache is excluded from the parameter cap, but its read/write traffic is included in memory bandwidth. Intermediate activations are excluded by the challenge convention. Attention MACs assume that the configured context buffer is fully populated; startup frames require less compute. FOV left is history, not latency; only FOV right contributes to algorithmic latency. STFT/ISTFT frames use centred hop alignment and have (FFT size - hop) / 2 samples of left and right context. Their overlap state remains FFT size - hop samples. Window and overlap-state bandwidth is shown explicitly in the first table row; FFT arithmetic is excluded.</t>
         </is>
       </c>
     </row>
@@ -3252,11 +3254,11 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ISTFT algorithmic latency (ms)</t>
+          <t>ISTFT synthesis lookahead (ms)</t>
         </is>
       </c>
       <c r="B15" s="3">
-        <f>($B$3-$B$4)/$B$2*1000</f>
+        <f>(($B$3-$B$4)/2)/$B$2*1000</f>
         <v/>
       </c>
     </row>
@@ -3454,18 +3456,20 @@
         <f>C20*L20</f>
         <v/>
       </c>
-      <c r="N20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="6" t="n">
-        <v>0</v>
+      <c r="N20" s="6">
+        <f>($B$3-$B$4)/2</f>
+        <v/>
+      </c>
+      <c r="O20" s="6">
+        <f>($B$3-$B$4)/2</f>
+        <v/>
       </c>
       <c r="P20" s="8">
-        <f>C20*N20/$B$5*1000</f>
+        <f>C20*N20/$B$2*1000</f>
         <v/>
       </c>
       <c r="Q20" s="8">
-        <f>C20*O20/$B$5*1000</f>
+        <f>C20*O20/$B$2*1000</f>
         <v/>
       </c>
       <c r="R20" s="7">
@@ -4907,7 +4911,7 @@
         <v/>
       </c>
       <c r="Q37" s="12">
-        <f>SUM(Q20:Q36)+$B$15</f>
+        <f>SUM(Q20:Q36)</f>
         <v/>
       </c>
       <c r="R37" s="12">
@@ -4962,7 +4966,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Memory bandwidth uses the bytes-per-value setting in B16 and includes model parameters, model buffers, convolution state, and attention KV-cache. Parameter-cap values include trainable parameters and non-runtime model buffers required for inference. Runtime state/cache is excluded from the parameter cap, but its read/write traffic is included in memory bandwidth. Intermediate activations are excluded by the challenge convention. Attention MACs assume that the configured context buffer is fully populated; startup frames require less compute. FOV left is history, not latency; only FOV right contributes to algorithmic latency. STFT/ISTFT window and overlap-state bandwidth is shown explicitly in the first table row; FFT arithmetic is excluded.</t>
+          <t>Memory bandwidth uses the bytes-per-value setting in B16 and includes model parameters, model buffers, convolution state, and attention KV-cache. Parameter-cap values include trainable parameters and non-runtime model buffers required for inference. Runtime state/cache is excluded from the parameter cap, but its read/write traffic is included in memory bandwidth. Intermediate activations are excluded by the challenge convention. Attention MACs assume that the configured context buffer is fully populated; startup frames require less compute. FOV left is history, not latency; only FOV right contributes to algorithmic latency. STFT/ISTFT frames use centred hop alignment and have (FFT size - hop) / 2 samples of left and right context. Their overlap state remains FFT size - hop samples. Window and overlap-state bandwidth is shown explicitly in the first table row; FFT arithmetic is excluded.</t>
         </is>
       </c>
     </row>

</xml_diff>